<commit_message>
Update Ocelli Finance data
</commit_message>
<xml_diff>
--- a/FINANCE.xlsx
+++ b/FINANCE.xlsx
@@ -428,29 +428,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>2</v>
+      <c r="A2" t="str">
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-15</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>asset</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>Bank Account</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>Opening Balance</v>
-      </c>
-      <c r="F2">
-        <v>719</v>
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Opening Balance</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>